<commit_message>
Update usn_list.xlsx to contain only 10 USNs by default
</commit_message>
<xml_diff>
--- a/usn_list.xlsx
+++ b/usn_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -423,6 +423,76 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1JT24IS001</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1JT24IS002</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>1JT24IS003</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>1JT24IS004</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>1JT24IS005</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1JT24IS006</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1JT24IS007</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>1JT24IS008</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>1JT24IS009</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>1JT24IS010</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>